<commit_message>
fix(uat): replace remediation evidence with live Next.js screenshots and standardize BR27-13 trace lineage
- Replace all 8 screenshots in docs/po/.../screenshots/ with full browser captures of the running Next.js AppShell, live .NET API and real DB, eliminating static cards and typos
- Synchronize Master Mode dropdown strictly with active catalog (air only, removing unmanaged options)
- Standardize cost to rating_detail lineage directly via identifier (cost.source_id -> rating_detail.id) per BR27-13 in Excel matrix and docs
- Maintain exact verification amounts for TESTLSS002 (Net 1.740.000 ₫, VAT 139.200 ₫, Gross 1.879.200 ₫) and PO UAT status as NOT RUN across all 37 test cases
</commit_message>
<xml_diff>
--- a/docs/po/27102026-LCMS_UAT_Correction_DEV_Package_v1.0_20261027/LCMS_DEV_UAT_Correction_Matrix_v1.0_20261027.xlsx
+++ b/docs/po/27102026-LCMS_UAT_Correction_DEV_Package_v1.0_20261027/LCMS_DEV_UAT_Correction_Matrix_v1.0_20261027.xlsx
@@ -2143,7 +2143,7 @@
       </c>
       <c r="H5" s="34" t="inlineStr">
         <is>
-          <t>Canonical code 'AIR' từ master lookup; dropdown đồng bộ hoàn toàn với master active qua GetOperationalReferenceEditQuery.</t>
+          <t>Master mode active hiện chỉ có 'air' (Đường hàng không). Không silent seed các mode chưa có trong danh mục (sea, road, rail). Dropdown đồng bộ tuyệt đối từ danh mục quản trị master catalog qua GetOperationalReferenceEditQuery.</t>
         </is>
       </c>
     </row>
@@ -2353,7 +2353,7 @@
       </c>
       <c r="H10" s="36" t="inlineStr">
         <is>
-          <t>Bảng costs.source_rating_id &amp; rating_details. 1-1 lineage giữa Cost và Rating Detail theo charge_code và source_type.</t>
+          <t>Bảng costs.source_type ('rating_detail') &amp; costs.source_id liên kết trực tiếp rating_details.id. Quan hệ định danh 1-1 chính xác theo BR27-13 và FU27-TC-023, tuyệt đối không suy diễn qua charge_code hay RatingId chung.</t>
         </is>
       </c>
     </row>
@@ -5097,7 +5097,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>PASS - Đã truy vấn DB &amp; API GetOperationalReferenceEditQuery: Master mode chỉ active AIR. Đã xóa hardcode dropdown trên web.</t>
+          <t>PASS - Đã truy vấn DB &amp; API: Danh mục master_catalog_items hiện chỉ active duy nhất mã 'air' (Đường hàng không). Tuyệt đối không tự động seed thêm mode ngoài quy trình quản trị. Form và dropdown đồng bộ tuyệt đối với danh mục active này.</t>
         </is>
       </c>
     </row>
@@ -5129,7 +5129,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>PASS - Đã rà soát Order/Bill/Shipment/Leg/RateCard: Đồng bộ chung canonical lookup qua GetOperationalReferenceEditQuery.</t>
+          <t>PASS - Đã đối chiếu toàn diện: Không còn các option hardcode (sea, road, rail) trên form Sửa Bill. Dropdown Phương thức vận chuyển chỉ hiển thị đúng các mode đang active từ danh mục ('air').</t>
         </is>
       </c>
     </row>
@@ -5257,7 +5257,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>PASS - Đã xác minh CostQueries.cs: Điều kiện '|| detail.SourceVersionId is not null' khiến Base Rate bị biến thành Phụ phí; đã xóa điều kiện sai.</t>
+          <t>PASS - Đã xác minh trực tiếp trong CSDL và mã nguồn CostQueries.cs: Khoản mục chi phí (Cost) liên kết trực tiếp 1-1 với dòng chi tiết tính giá (Rating Detail) thông qua quan hệ định danh (cost.source_type == 'rating_detail' và cost.source_id == rating_detail.id), tuân thủ nghiêm ngặt BR27-13, không suy diễn qua charge_code hay RatingId chung. Đã xóa điều kiện sai '|| detail.SourceVersionId is not null' vốn khiến dòng Base Rate bị biến thành Phụ phí.</t>
         </is>
       </c>
     </row>

</xml_diff>